<commit_message>
Philippine geography and practice masters out of the box: PSGC regions, provinces, cities and municipalities, ZIP codes, barangay loader; Province replaces State; Thai reference rows retired
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/Bank_Upload_Template.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/Bank_Upload_Template.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="81">
   <si>
     <t xml:space="preserve">Bank Code</t>
   </si>
@@ -24,7 +24,7 @@
     <t xml:space="preserve">Bank Branch</t>
   </si>
   <si>
-    <t xml:space="preserve">IFSC / SWIFT Code</t>
+    <t xml:space="preserve">SWIFT Code</t>
   </si>
   <si>
     <t xml:space="preserve">Address Line 1</t>
@@ -36,114 +36,117 @@
     <t xml:space="preserve">Address Line 3</t>
   </si>
   <si>
+    <t xml:space="preserve">City / Municipality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Province</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CITI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citibank, N.A. (Philippine Branch)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bonifacio Global City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CITIPHMX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 Bonifacio High Street, 5th Ave.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taguig City</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metro Manila</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Philippines</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+63 2 8995 9999</t>
+  </si>
+  <si>
+    <t xml:space="preserve">customer.service@citi.example.ph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commercial Bank</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Column</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Allowed values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Other accepted headers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bankCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bankName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bankBranch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SWIFT / BIC code of the branch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ifscCode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AddressLine1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AddressLine2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AddressLine3</t>
+  </si>
+  <si>
     <t xml:space="preserve">City</t>
   </si>
   <si>
-    <t xml:space="preserve">State</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Country</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UBP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Union Bank of the Philippines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ortigas Center</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UBPHPHMM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UnionBank Plaza, Meralco Ave.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pasig</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Metro Manila</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Philippines</t>
-  </si>
-  <si>
-    <t xml:space="preserve">+63 2 8841 8600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">customer.service@unionbank.example.ph</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Universal Bank</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Column</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Required</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Allowed values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Example</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Other accepted headers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bankCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bankName</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bankBranch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SWIFT / BIC code of the branch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ifscCode</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AddressLine1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AddressLine2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AddressLine3</t>
-  </si>
-  <si>
     <t xml:space="preserve">state</t>
   </si>
   <si>
@@ -213,7 +216,7 @@
     <t xml:space="preserve">Required columns</t>
   </si>
   <si>
-    <t xml:space="preserve">Bank Code, Bank Name, Bank Branch, IFSC / SWIFT Code, City, State, Country, Phone, Email ID (dark red headers on the Data sheet). Other columns may be left empty or removed.</t>
+    <t xml:space="preserve">Bank Code, Bank Name, Bank Branch, SWIFT Code, City / Municipality, Province, Country, Phone, Email ID (dark red headers on the Data sheet). Other columns may be left empty or removed.</t>
   </si>
   <si>
     <t xml:space="preserve">Header row</t>
@@ -244,6 +247,9 @@
   </si>
   <si>
     <t xml:space="preserve">Each row creates a new record, checked exactly like Add on the screen. A row whose code already exists is refused (edit existing records on the screen).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The main Philippine banks are shipped (BDO, BPI, Metrobank, Land Bank, PNB, Security Bank, UnionBank, RCBC, China Bank, EastWest, DBP, PSBank, AUB, Maybank, PBCom, Bank of Commerce, Veterans Bank) with their SWIFT codes. Add the others you deal with.</t>
   </si>
   <si>
     <t xml:space="preserve">Source</t>
@@ -384,11 +390,11 @@
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="23" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="14" customWidth="1"/>
@@ -644,6 +650,9 @@
       <c r="E9" s="0" t="s">
         <v>20</v>
       </c>
+      <c r="F9" s="4" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
@@ -659,7 +668,7 @@
         <v>21</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
@@ -690,7 +699,7 @@
         <v>23</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13">
@@ -712,13 +721,13 @@
         <v>32</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E14" s="0" t="s">
         <v>24</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
@@ -729,16 +738,16 @@
         <v>39</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E15" s="0" t="s">
         <v>25</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
@@ -749,13 +758,13 @@
         <v>39</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -765,7 +774,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -774,106 +783,111 @@
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="0" t="s">
-        <v>77</v>
-      </c>
       <c r="B13" s="4" t="s">
         <v>78</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>